<commit_message>
Sửa lỗi User agent quá dài và Newsletter email rỗng
</commit_message>
<xml_diff>
--- a/Từ khóa.xlsx
+++ b/Từ khóa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\Laravel\xanhworld.vn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA51FF78-BBB3-4F06-B178-9B7F210D9966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F9917A6-6F53-4E5E-B0F6-CA477812880C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="204" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="271">
   <si>
     <t>cây kim tiền</t>
   </si>
@@ -821,6 +821,21 @@
   </si>
   <si>
     <t>cau trắng</t>
+  </si>
+  <si>
+    <t>https://xanhworld.vn/san-pham/cay-cau-trang-gia-tot-cung-cap-cay-cong-trinh-toan-quoc</t>
+  </si>
+  <si>
+    <t>https://xanhworld.vn/san-pham/cay-luoi-ho-y-nghia-phong-thuy-cach-cham-soc-cong-dung</t>
+  </si>
+  <si>
+    <t>https://xanhworld.vn/san-pham/cay-hanh-phuc-phong-thuy-cay-canh-noi-that-cao-cap</t>
+  </si>
+  <si>
+    <t>https://xanhworld.vn/san-pham/cay-hoa-giay-trang-tri-cay-leo-gian-dep-de-trong</t>
+  </si>
+  <si>
+    <t>https://xanhworld.vn/san-pham/cay-cha-la-canh-cay-trang-tri-san-vuon-cao-cap</t>
   </si>
 </sst>
 </file>
@@ -1303,6 +1318,9 @@
       <c r="B4" s="2">
         <v>33100</v>
       </c>
+      <c r="C4" s="2" t="s">
+        <v>266</v>
+      </c>
     </row>
     <row r="5" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -1322,6 +1340,9 @@
       <c r="B6" s="2">
         <v>27100</v>
       </c>
+      <c r="C6" s="2" t="s">
+        <v>268</v>
+      </c>
     </row>
     <row r="7" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -1330,6 +1351,9 @@
       <c r="B7" s="2">
         <v>22200</v>
       </c>
+      <c r="C7" s="2" t="s">
+        <v>267</v>
+      </c>
     </row>
     <row r="8" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -1338,6 +1362,9 @@
       <c r="B8" s="2">
         <v>18100</v>
       </c>
+      <c r="C8" s="2" t="s">
+        <v>269</v>
+      </c>
     </row>
     <row r="9" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -1345,6 +1372,9 @@
       </c>
       <c r="B9" s="2">
         <v>18100</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>